<commit_message>
Controle de entrega: 1º romaneio Sabagram (210 placas, 167,93 m²)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0176EKqwb7amr9sfwoHiH6NW
</commit_message>
<xml_diff>
--- a/Controle_Entrega_Granito_Ed_Jardim.xlsx
+++ b/Controle_Entrega_Granito_Ed_Jardim.xlsx
@@ -33,12 +33,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -137,6 +138,10 @@
       <sz val="10"/>
       <name val="Aptos Narrow"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -210,7 +215,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -450,11 +455,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="D0D5D8"/>
+      </left>
+      <right style="thin">
+        <color rgb="D0D5D8"/>
+      </right>
+      <top style="thin">
+        <color rgb="D0D5D8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="D0D5D8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -512,7 +532,10 @@
     <xf numFmtId="0" fontId="19" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4173,7 +4196,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G20"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -4254,26 +4277,348 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="str">
-        <v>(sem recebimentos registrados)</v>
-      </c>
-      <c r="B5" s="21" t="str">
-        <v/>
-      </c>
-      <c r="C5" s="21" t="str">
-        <v/>
-      </c>
-      <c r="D5" s="21" t="str">
-        <v/>
-      </c>
-      <c r="E5" s="21" t="str">
-        <v/>
-      </c>
-      <c r="F5" s="21" t="str">
-        <v/>
-      </c>
-      <c r="G5" s="21" t="str">
-        <v/>
+      <c r="A5" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B5" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C5" s="11" t="str">
+        <v>C3</v>
+      </c>
+      <c r="D5" s="11">
+        <v>22</v>
+      </c>
+      <c r="E5" s="11">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13">
+        <f>D5*INDEX('ODC-300'!$L$5:$L$80,MATCH(C5,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G5" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B6" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C6" s="11" t="str">
+        <v>C4</v>
+      </c>
+      <c r="D6" s="11">
+        <v>44</v>
+      </c>
+      <c r="E6" s="11">
+        <v>0</v>
+      </c>
+      <c r="F6" s="13">
+        <f>D6*INDEX('ODC-300'!$L$5:$L$80,MATCH(C6,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G6" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B7" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C7" s="11" t="str">
+        <v>C5</v>
+      </c>
+      <c r="D7" s="11">
+        <v>22</v>
+      </c>
+      <c r="E7" s="11">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13">
+        <f>D7*INDEX('ODC-300'!$L$5:$L$80,MATCH(C7,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G7" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B8" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C8" s="11" t="str">
+        <v>C7</v>
+      </c>
+      <c r="D8" s="11">
+        <v>4</v>
+      </c>
+      <c r="E8" s="11">
+        <v>0</v>
+      </c>
+      <c r="F8" s="13">
+        <f>D8*INDEX('ODC-300'!$L$5:$L$80,MATCH(C8,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G8" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B9" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C9" s="11" t="str">
+        <v>C15</v>
+      </c>
+      <c r="D9" s="11">
+        <v>96</v>
+      </c>
+      <c r="E9" s="11">
+        <v>0</v>
+      </c>
+      <c r="F9" s="13">
+        <f>D9*INDEX('ODC-300'!$L$5:$L$80,MATCH(C9,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G9" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B10" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C10" s="11" t="str">
+        <v>C17</v>
+      </c>
+      <c r="D10" s="11">
+        <v>2</v>
+      </c>
+      <c r="E10" s="11">
+        <v>0</v>
+      </c>
+      <c r="F10" s="13">
+        <f>D10*INDEX('ODC-300'!$L$5:$L$80,MATCH(C10,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G10" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B11" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C11" s="11" t="str">
+        <v>C18</v>
+      </c>
+      <c r="D11" s="11">
+        <v>2</v>
+      </c>
+      <c r="E11" s="11">
+        <v>0</v>
+      </c>
+      <c r="F11" s="13">
+        <f>D11*INDEX('ODC-300'!$L$5:$L$80,MATCH(C11,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G11" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B12" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C12" s="11" t="str">
+        <v>C19</v>
+      </c>
+      <c r="D12" s="11">
+        <v>2</v>
+      </c>
+      <c r="E12" s="11">
+        <v>0</v>
+      </c>
+      <c r="F12" s="13">
+        <f>D12*INDEX('ODC-300'!$L$5:$L$80,MATCH(C12,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G12" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B13" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C13" s="11" t="str">
+        <v>C21</v>
+      </c>
+      <c r="D13" s="11">
+        <v>2</v>
+      </c>
+      <c r="E13" s="11">
+        <v>0</v>
+      </c>
+      <c r="F13" s="13">
+        <f>D13*INDEX('ODC-300'!$L$5:$L$80,MATCH(C13,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G13" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B14" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C14" s="11" t="str">
+        <v>C25</v>
+      </c>
+      <c r="D14" s="11">
+        <v>1</v>
+      </c>
+      <c r="E14" s="11">
+        <v>0</v>
+      </c>
+      <c r="F14" s="13">
+        <f>D14*INDEX('ODC-300'!$L$5:$L$80,MATCH(C14,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G14" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B15" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C15" s="11" t="str">
+        <v>C27</v>
+      </c>
+      <c r="D15" s="11">
+        <v>1</v>
+      </c>
+      <c r="E15" s="11">
+        <v>0</v>
+      </c>
+      <c r="F15" s="13">
+        <f>D15*INDEX('ODC-300'!$L$5:$L$80,MATCH(C15,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G15" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B16" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C16" s="11" t="str">
+        <v>C28</v>
+      </c>
+      <c r="D16" s="11">
+        <v>1</v>
+      </c>
+      <c r="E16" s="11">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13">
+        <f>D16*INDEX('ODC-300'!$L$5:$L$80,MATCH(C16,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G16" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B17" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C17" s="11" t="str">
+        <v>C29</v>
+      </c>
+      <c r="D17" s="11">
+        <v>2</v>
+      </c>
+      <c r="E17" s="11">
+        <v>0</v>
+      </c>
+      <c r="F17" s="13">
+        <f>D17*INDEX('ODC-300'!$L$5:$L$80,MATCH(C17,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G17" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B18" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C18" s="11" t="str">
+        <v>C30</v>
+      </c>
+      <c r="D18" s="11">
+        <v>6</v>
+      </c>
+      <c r="E18" s="11">
+        <v>0</v>
+      </c>
+      <c r="F18" s="13">
+        <f>D18*INDEX('ODC-300'!$L$5:$L$80,MATCH(C18,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G18" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21">
+        <v>46290</v>
+      </c>
+      <c r="B19" s="22" t="str">
+        <v>Romaneio Sabagram · emissão 15/09/2026</v>
+      </c>
+      <c r="C19" s="11" t="str">
+        <v>C31</v>
+      </c>
+      <c r="D19" s="11">
+        <v>3</v>
+      </c>
+      <c r="E19" s="11">
+        <v>0</v>
+      </c>
+      <c r="F19" s="13">
+        <f>D19*INDEX('ODC-300'!$L$5:$L$80,MATCH(C19,'ODC-300'!$A$5:$A$80,0))</f>
+      </c>
+      <c r="G19" s="22" t="str">
+        <v>Carregamento 25/09/2026 · 8 paletes (P1–P8) · material descrito como "Cinza Mundo Novo Bruto" · C4: paletes P6=23 + P7=22 somam 45, romaneio informa 44</v>
       </c>
     </row>
   </sheetData>
@@ -4282,7 +4627,7 @@
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>